<commit_message>
Make the overview KPI block render consistently
The overview's conditional formatting still covered only rows 6-17, so the
2029, 2030 and total blocks appeared unhighlighted while the earlier ones
were colored. The range now follows the block, and the charts label every
third month so 54 categories stay readable.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USZ2QFd3neqnzoYuSHpCqM
</commit_message>
<xml_diff>
--- a/deliverables/cashflow/20260817_Cashflow_SmartInfra_DusL.xlsx
+++ b/deliverables/cashflow/20260817_Cashflow_SmartInfra_DusL.xlsx
@@ -5196,6 +5196,8 @@
         <minorTickMark val="none"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="3"/>
+        <tickMarkSkip val="3"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -5338,6 +5340,8 @@
         <minorTickMark val="none"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="3"/>
+        <tickMarkSkip val="3"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -6202,7 +6206,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:B17">
+  <conditionalFormatting sqref="B6:B29">
     <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="9">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Fix the overview charts' axes and line rendering
The category axis was written as a left-hand axis and its labels were drawn
at the axis crossing, so with negative months they ran through the middle of
the plot. Both charts now place the category axis at the bottom with labels
below it, keep their axes visible, and draw straight segments instead of
splines, which misrepresented a cumulative series.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USZ2QFd3neqnzoYuSHpCqM
</commit_message>
<xml_diff>
--- a/deliverables/cashflow/20260817_Cashflow_SmartInfra_DusL.xlsx
+++ b/deliverables/cashflow/20260817_Cashflow_SmartInfra_DusL.xlsx
@@ -5182,7 +5182,8 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="40"/>
+        <gapWidth val="60"/>
+        <overlap val="-10"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -5191,9 +5192,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
         <tickLblSkip val="3"/>
@@ -5204,6 +5207,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -5222,8 +5226,9 @@
           </tx>
         </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -5291,6 +5296,7 @@
               <f>'Cashflow'!$C$78:$BD$78</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -5326,6 +5332,7 @@
               <f>'Cashflow'!$C$79:$BD$79</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -5335,9 +5342,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
         <tickLblSkip val="3"/>
@@ -5348,6 +5357,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -5366,8 +5376,9 @@
           </tx>
         </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -5389,7 +5400,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10800000" cy="2880000"/>
+    <ext cx="11520000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -5411,7 +5422,7 @@
       <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10800000" cy="2880000"/>
+    <ext cx="11520000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>

<commit_message>
Give the overview KPI table a continuous background
The label column carried no fill, so with gridlines off the table read as
floating text rather than a block. Label cells now take the same fill as
their value cell, and both charts get an explicit white area with a light
border instead of a transparent one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USZ2QFd3neqnzoYuSHpCqM
</commit_message>
<xml_diff>
--- a/deliverables/cashflow/20260817_Cashflow_SmartInfra_DusL.xlsx
+++ b/deliverables/cashflow/20260817_Cashflow_SmartInfra_DusL.xlsx
@@ -229,7 +229,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -270,6 +270,16 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.3499862666707358"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -489,7 +499,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -623,6 +633,12 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="28" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="167" fontId="13" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment indent="1"/>
+    </xf>
     <xf numFmtId="167" fontId="28" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="167" fontId="28" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -5238,6 +5254,17 @@
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="BFBFBF"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -5388,6 +5415,17 @@
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="BFBFBF"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -5979,7 +6017,7 @@
       <c r="B6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="95" t="inlineStr">
         <is>
           <t>Einnahmen H2 2026</t>
         </is>
@@ -5990,7 +6028,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="95" t="inlineStr">
         <is>
           <t>Ausgaben H2 2026</t>
         </is>
@@ -6001,7 +6039,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="96" t="inlineStr">
         <is>
           <t>Netto-Cashflow H2 2026</t>
         </is>
@@ -6020,7 +6058,7 @@
       <c r="B10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="95" t="inlineStr">
         <is>
           <t>Einnahmen 2027</t>
         </is>
@@ -6031,7 +6069,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="95" t="inlineStr">
         <is>
           <t>Ausgaben 2027</t>
         </is>
@@ -6042,7 +6080,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="96" t="inlineStr">
         <is>
           <t>Netto-Cashflow 2027</t>
         </is>
@@ -6061,7 +6099,7 @@
       <c r="B14" s="7" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="95" t="inlineStr">
         <is>
           <t>Einnahmen 2028</t>
         </is>
@@ -6072,7 +6110,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="95" t="inlineStr">
         <is>
           <t>Ausgaben 2028</t>
         </is>
@@ -6083,7 +6121,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="96" t="inlineStr">
         <is>
           <t>Netto-Cashflow 2028</t>
         </is>
@@ -6102,7 +6140,7 @@
       <c r="B18" s="7" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="95" t="inlineStr">
         <is>
           <t>Einnahmen 2029</t>
         </is>
@@ -6113,7 +6151,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="95" t="inlineStr">
         <is>
           <t>Ausgaben 2029</t>
         </is>
@@ -6124,7 +6162,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="96" t="inlineStr">
         <is>
           <t>Netto-Cashflow 2029</t>
         </is>
@@ -6143,7 +6181,7 @@
       <c r="B22" s="7" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="95" t="inlineStr">
         <is>
           <t>Einnahmen 2030</t>
         </is>
@@ -6154,7 +6192,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="95" t="inlineStr">
         <is>
           <t>Ausgaben 2030</t>
         </is>
@@ -6165,7 +6203,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="96" t="inlineStr">
         <is>
           <t>Netto-Cashflow 2030</t>
         </is>
@@ -6184,7 +6222,7 @@
       <c r="B26" s="7" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="A27" s="95" t="inlineStr">
         <is>
           <t>Gesamteinnahmen</t>
         </is>
@@ -6195,7 +6233,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="A28" s="95" t="inlineStr">
         <is>
           <t>Gesamtausgaben</t>
         </is>
@@ -6206,7 +6244,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="96" t="inlineStr">
         <is>
           <t>Gesamt-Netto-Cashflow</t>
         </is>
@@ -41988,11 +42026,11 @@
         </is>
       </c>
       <c r="F7" s="28" t="n"/>
-      <c r="G7" s="95" t="n">
+      <c r="G7" s="97" t="n">
         <v>2551.74</v>
       </c>
       <c r="H7" s="24" t="n"/>
-      <c r="I7" s="96" t="n">
+      <c r="I7" s="98" t="n">
         <v>11392.81</v>
       </c>
       <c r="J7" s="26" t="n">
@@ -42033,11 +42071,11 @@
         </is>
       </c>
       <c r="F8" s="28" t="n"/>
-      <c r="G8" s="95" t="n">
+      <c r="G8" s="97" t="n">
         <v>5327.69</v>
       </c>
       <c r="H8" s="24" t="n"/>
-      <c r="I8" s="96" t="n">
+      <c r="I8" s="98" t="n">
         <v>17939.49</v>
       </c>
       <c r="J8" s="26" t="n">
@@ -42078,9 +42116,9 @@
         </is>
       </c>
       <c r="F9" s="28" t="n"/>
-      <c r="G9" s="95" t="n"/>
+      <c r="G9" s="97" t="n"/>
       <c r="H9" s="24" t="n"/>
-      <c r="I9" s="96" t="n"/>
+      <c r="I9" s="98" t="n"/>
       <c r="J9" s="26" t="n">
         <v>1</v>
       </c>
@@ -42119,11 +42157,11 @@
         </is>
       </c>
       <c r="F10" s="28" t="n"/>
-      <c r="G10" s="95" t="n"/>
+      <c r="G10" s="97" t="n"/>
       <c r="H10" s="24" t="n">
         <v>46295</v>
       </c>
-      <c r="I10" s="96" t="n">
+      <c r="I10" s="98" t="n">
         <v>600</v>
       </c>
       <c r="J10" s="26" t="n">
@@ -42168,9 +42206,9 @@
         </is>
       </c>
       <c r="F11" s="28" t="n"/>
-      <c r="G11" s="95" t="n"/>
+      <c r="G11" s="97" t="n"/>
       <c r="H11" s="24" t="n"/>
-      <c r="I11" s="96" t="n">
+      <c r="I11" s="98" t="n">
         <v>31807.45</v>
       </c>
       <c r="J11" s="26" t="n">
@@ -42213,13 +42251,13 @@
       <c r="F12" s="28" t="n">
         <v>46280</v>
       </c>
-      <c r="G12" s="95" t="n">
+      <c r="G12" s="97" t="n">
         <v>5400</v>
       </c>
       <c r="H12" s="24" t="n">
         <v>46341</v>
       </c>
-      <c r="I12" s="96" t="n">
+      <c r="I12" s="98" t="n">
         <v>15594.65</v>
       </c>
       <c r="J12" s="26" t="n">
@@ -42264,11 +42302,11 @@
         </is>
       </c>
       <c r="F13" s="28" t="n"/>
-      <c r="G13" s="95" t="n"/>
+      <c r="G13" s="97" t="n"/>
       <c r="H13" s="24" t="n">
         <v>46310</v>
       </c>
-      <c r="I13" s="96" t="n">
+      <c r="I13" s="98" t="n">
         <v>60000</v>
       </c>
       <c r="J13" s="26" t="n">
@@ -42313,9 +42351,9 @@
         </is>
       </c>
       <c r="F14" s="28" t="n"/>
-      <c r="G14" s="95" t="n"/>
+      <c r="G14" s="97" t="n"/>
       <c r="H14" s="24" t="n"/>
-      <c r="I14" s="96" t="n">
+      <c r="I14" s="98" t="n">
         <v>29760</v>
       </c>
       <c r="J14" s="26" t="n">
@@ -42356,9 +42394,9 @@
         </is>
       </c>
       <c r="F15" s="28" t="n"/>
-      <c r="G15" s="95" t="n"/>
+      <c r="G15" s="97" t="n"/>
       <c r="H15" s="24" t="n"/>
-      <c r="I15" s="96" t="n">
+      <c r="I15" s="98" t="n">
         <v>27750</v>
       </c>
       <c r="J15" s="26" t="n">
@@ -42399,9 +42437,9 @@
         </is>
       </c>
       <c r="F16" s="28" t="n"/>
-      <c r="G16" s="97" t="n"/>
+      <c r="G16" s="99" t="n"/>
       <c r="H16" s="24" t="n"/>
-      <c r="I16" s="96" t="n">
+      <c r="I16" s="98" t="n">
         <v>14970</v>
       </c>
       <c r="J16" s="26" t="n">
@@ -42446,9 +42484,9 @@
         </is>
       </c>
       <c r="F17" s="28" t="n"/>
-      <c r="G17" s="95" t="n"/>
+      <c r="G17" s="97" t="n"/>
       <c r="H17" s="24" t="n"/>
-      <c r="I17" s="96" t="n"/>
+      <c r="I17" s="98" t="n"/>
       <c r="J17" s="26" t="n">
         <v>1</v>
       </c>
@@ -42491,9 +42529,9 @@
         </is>
       </c>
       <c r="F18" s="28" t="n"/>
-      <c r="G18" s="95" t="n"/>
+      <c r="G18" s="97" t="n"/>
       <c r="H18" s="24" t="n"/>
-      <c r="I18" s="96" t="n"/>
+      <c r="I18" s="98" t="n"/>
       <c r="J18" s="26" t="n">
         <v>1</v>
       </c>
@@ -42536,9 +42574,9 @@
         </is>
       </c>
       <c r="F19" s="28" t="n"/>
-      <c r="G19" s="95" t="n"/>
+      <c r="G19" s="97" t="n"/>
       <c r="H19" s="24" t="n"/>
-      <c r="I19" s="96" t="n"/>
+      <c r="I19" s="98" t="n"/>
       <c r="J19" s="26" t="n">
         <v>1</v>
       </c>
@@ -42581,9 +42619,9 @@
         </is>
       </c>
       <c r="F20" s="28" t="n"/>
-      <c r="G20" s="95" t="n"/>
+      <c r="G20" s="97" t="n"/>
       <c r="H20" s="24" t="n"/>
-      <c r="I20" s="96" t="n"/>
+      <c r="I20" s="98" t="n"/>
       <c r="J20" s="26" t="n">
         <v>1</v>
       </c>
@@ -42626,9 +42664,9 @@
         </is>
       </c>
       <c r="F21" s="28" t="n"/>
-      <c r="G21" s="95" t="n"/>
+      <c r="G21" s="97" t="n"/>
       <c r="H21" s="24" t="n"/>
-      <c r="I21" s="96" t="n">
+      <c r="I21" s="98" t="n">
         <v>29750</v>
       </c>
       <c r="J21" s="26" t="n">
@@ -42669,9 +42707,9 @@
         </is>
       </c>
       <c r="F22" s="28" t="n"/>
-      <c r="G22" s="95" t="n"/>
+      <c r="G22" s="97" t="n"/>
       <c r="H22" s="24" t="n"/>
-      <c r="I22" s="96" t="n">
+      <c r="I22" s="98" t="n">
         <v>9750</v>
       </c>
       <c r="J22" s="26" t="n">
@@ -42714,13 +42752,13 @@
       <c r="F23" s="28" t="n">
         <v>46402</v>
       </c>
-      <c r="G23" s="95" t="n">
+      <c r="G23" s="97" t="n">
         <v>5000</v>
       </c>
       <c r="H23" s="24" t="n">
         <v>46433</v>
       </c>
-      <c r="I23" s="96" t="n">
+      <c r="I23" s="98" t="n">
         <v>6590.1</v>
       </c>
       <c r="J23" s="26" t="n">
@@ -42761,9 +42799,9 @@
         </is>
       </c>
       <c r="F24" s="28" t="n"/>
-      <c r="G24" s="95" t="n"/>
+      <c r="G24" s="97" t="n"/>
       <c r="H24" s="24" t="n"/>
-      <c r="I24" s="96" t="n">
+      <c r="I24" s="98" t="n">
         <v>13996.4</v>
       </c>
       <c r="J24" s="26" t="n">
@@ -42808,9 +42846,9 @@
         </is>
       </c>
       <c r="F25" s="28" t="n"/>
-      <c r="G25" s="95" t="n"/>
+      <c r="G25" s="97" t="n"/>
       <c r="H25" s="24" t="n"/>
-      <c r="I25" s="96" t="n">
+      <c r="I25" s="98" t="n">
         <v>17133.62</v>
       </c>
       <c r="J25" s="26" t="n">
@@ -42855,9 +42893,9 @@
         </is>
       </c>
       <c r="F26" s="28" t="n"/>
-      <c r="G26" s="95" t="n"/>
+      <c r="G26" s="97" t="n"/>
       <c r="H26" s="24" t="n"/>
-      <c r="I26" s="96" t="n">
+      <c r="I26" s="98" t="n">
         <v>620</v>
       </c>
       <c r="J26" s="26" t="n">
@@ -42900,14 +42938,14 @@
       <c r="F27" s="28" t="n">
         <v>46440</v>
       </c>
-      <c r="G27" s="95">
+      <c r="G27" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
       <c r="H27" s="24" t="n">
         <v>46583</v>
       </c>
-      <c r="I27" s="96" t="n">
+      <c r="I27" s="98" t="n">
         <v>83828.39999999999</v>
       </c>
       <c r="J27" s="26" t="n">
@@ -42950,7 +42988,7 @@
       <c r="F28" s="91" t="n">
         <v>46517</v>
       </c>
-      <c r="G28" s="95" t="n">
+      <c r="G28" s="97" t="n">
         <v>163443.6</v>
       </c>
       <c r="H28" s="24">
@@ -42958,7 +42996,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I28" s="96" t="n">
+      <c r="I28" s="98" t="n">
         <v>222875.03</v>
       </c>
       <c r="J28" s="26" t="n">
@@ -43001,7 +43039,7 @@
       <c r="F29" s="91" t="n">
         <v>46608</v>
       </c>
-      <c r="G29" s="95" t="n">
+      <c r="G29" s="97" t="n">
         <v>149917.66</v>
       </c>
       <c r="H29" s="24">
@@ -43009,7 +43047,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I29" s="96" t="n">
+      <c r="I29" s="98" t="n">
         <v>205494.2</v>
       </c>
       <c r="J29" s="26" t="n">
@@ -43052,7 +43090,7 @@
       <c r="F30" s="91" t="n">
         <v>46622</v>
       </c>
-      <c r="G30" s="95" t="n">
+      <c r="G30" s="97" t="n">
         <v>41710.17</v>
       </c>
       <c r="H30" s="24">
@@ -43060,7 +43098,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I30" s="96" t="n">
+      <c r="I30" s="98" t="n">
         <v>66447.57000000001</v>
       </c>
       <c r="J30" s="26" t="n">
@@ -43103,7 +43141,7 @@
       <c r="F31" s="91" t="n">
         <v>46650</v>
       </c>
-      <c r="G31" s="95" t="n">
+      <c r="G31" s="97" t="n">
         <v>109339.85</v>
       </c>
       <c r="H31" s="24">
@@ -43111,7 +43149,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I31" s="96" t="n">
+      <c r="I31" s="98" t="n">
         <v>153351.72</v>
       </c>
       <c r="J31" s="26" t="n">
@@ -43154,7 +43192,7 @@
       <c r="F32" s="91" t="n">
         <v>46664</v>
       </c>
-      <c r="G32" s="95" t="n">
+      <c r="G32" s="97" t="n">
         <v>68762.03999999999</v>
       </c>
       <c r="H32" s="24">
@@ -43162,7 +43200,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I32" s="96" t="n">
+      <c r="I32" s="98" t="n">
         <v>101209.23</v>
       </c>
       <c r="J32" s="26" t="n">
@@ -43205,7 +43243,7 @@
       <c r="F33" s="91" t="n">
         <v>46797</v>
       </c>
-      <c r="G33" s="95" t="n">
+      <c r="G33" s="97" t="n">
         <v>68762.03999999999</v>
       </c>
       <c r="H33" s="24">
@@ -43213,7 +43251,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I33" s="96" t="n">
+      <c r="I33" s="98" t="n">
         <v>101209.23</v>
       </c>
       <c r="J33" s="26" t="n">
@@ -43256,7 +43294,7 @@
       <c r="F34" s="91" t="n">
         <v>46811</v>
       </c>
-      <c r="G34" s="95">
+      <c r="G34" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43265,7 +43303,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I34" s="96" t="n">
+      <c r="I34" s="98" t="n">
         <v>66447.57000000001</v>
       </c>
       <c r="J34" s="26" t="n">
@@ -43308,7 +43346,7 @@
       <c r="F35" s="91" t="n">
         <v>46818</v>
       </c>
-      <c r="G35" s="95">
+      <c r="G35" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43317,7 +43355,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I35" s="96" t="n">
+      <c r="I35" s="98" t="n">
         <v>66447.57000000001</v>
       </c>
       <c r="J35" s="26" t="n">
@@ -43360,7 +43398,7 @@
       <c r="F36" s="91" t="n">
         <v>46881</v>
       </c>
-      <c r="G36" s="95">
+      <c r="G36" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43369,7 +43407,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I36" s="96" t="n">
+      <c r="I36" s="98" t="n">
         <v>188113.37</v>
       </c>
       <c r="J36" s="26" t="n">
@@ -43412,7 +43450,7 @@
       <c r="F37" s="91" t="n">
         <v>46888</v>
       </c>
-      <c r="G37" s="95">
+      <c r="G37" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43421,7 +43459,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I37" s="96" t="n">
+      <c r="I37" s="98" t="n">
         <v>66447.57000000001</v>
       </c>
       <c r="J37" s="26" t="n">
@@ -43464,7 +43502,7 @@
       <c r="F38" s="91" t="n">
         <v>47126</v>
       </c>
-      <c r="G38" s="95">
+      <c r="G38" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43473,7 +43511,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I38" s="96" t="n">
+      <c r="I38" s="98" t="n">
         <v>118590.06</v>
       </c>
       <c r="J38" s="26" t="n">
@@ -43516,7 +43554,7 @@
       <c r="F39" s="91" t="n">
         <v>47196</v>
       </c>
-      <c r="G39" s="95">
+      <c r="G39" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43525,7 +43563,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I39" s="96" t="n">
+      <c r="I39" s="98" t="n">
         <v>101209.23</v>
       </c>
       <c r="J39" s="26" t="n">
@@ -43568,7 +43606,7 @@
       <c r="F40" s="91" t="n">
         <v>47315</v>
       </c>
-      <c r="G40" s="95" t="n">
+      <c r="G40" s="97" t="n">
         <v>163443.6</v>
       </c>
       <c r="H40" s="24">
@@ -43576,7 +43614,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I40" s="96" t="n">
+      <c r="I40" s="98" t="n">
         <v>222875.03</v>
       </c>
       <c r="J40" s="26" t="n">
@@ -43619,7 +43657,7 @@
       <c r="F41" s="91" t="n">
         <v>47196</v>
       </c>
-      <c r="G41" s="95">
+      <c r="G41" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43628,7 +43666,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I41" s="96" t="n">
+      <c r="I41" s="98" t="n">
         <v>66447.57000000001</v>
       </c>
       <c r="J41" s="26" t="n">
@@ -43671,7 +43709,7 @@
       <c r="F42" s="91" t="n">
         <v>47357</v>
       </c>
-      <c r="G42" s="95">
+      <c r="G42" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43680,7 +43718,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I42" s="96" t="n">
+      <c r="I42" s="98" t="n">
         <v>83828.39999999999</v>
       </c>
       <c r="J42" s="26" t="n">
@@ -43723,7 +43761,7 @@
       <c r="F43" s="91" t="n">
         <v>47546</v>
       </c>
-      <c r="G43" s="95">
+      <c r="G43" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43732,7 +43770,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I43" s="96" t="n">
+      <c r="I43" s="98" t="n">
         <v>83828.39999999999</v>
       </c>
       <c r="J43" s="26" t="n">
@@ -43775,7 +43813,7 @@
       <c r="F44" s="91" t="n">
         <v>47546</v>
       </c>
-      <c r="G44" s="95">
+      <c r="G44" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43784,7 +43822,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I44" s="96" t="n">
+      <c r="I44" s="98" t="n">
         <v>222875.03</v>
       </c>
       <c r="J44" s="26" t="n">
@@ -43827,7 +43865,7 @@
       <c r="F45" s="91" t="n">
         <v>47567</v>
       </c>
-      <c r="G45" s="95">
+      <c r="G45" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43836,7 +43874,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I45" s="96" t="n">
+      <c r="I45" s="98" t="n">
         <v>101209.23</v>
       </c>
       <c r="J45" s="26" t="n">
@@ -43879,7 +43917,7 @@
       <c r="F46" s="91" t="n">
         <v>47588</v>
       </c>
-      <c r="G46" s="95">
+      <c r="G46" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43888,7 +43926,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I46" s="96" t="n">
+      <c r="I46" s="98" t="n">
         <v>101209.23</v>
       </c>
       <c r="J46" s="26" t="n">
@@ -43931,7 +43969,7 @@
       <c r="F47" s="91" t="n">
         <v>47588</v>
       </c>
-      <c r="G47" s="95">
+      <c r="G47" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43940,7 +43978,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I47" s="96" t="n">
+      <c r="I47" s="98" t="n">
         <v>118590.06</v>
       </c>
       <c r="J47" s="26" t="n">
@@ -43983,7 +44021,7 @@
       <c r="F48" s="91" t="n">
         <v>47588</v>
       </c>
-      <c r="G48" s="95">
+      <c r="G48" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -43992,7 +44030,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I48" s="96" t="n">
+      <c r="I48" s="98" t="n">
         <v>135970.89</v>
       </c>
       <c r="J48" s="26" t="n">
@@ -44035,7 +44073,7 @@
       <c r="F49" s="91" t="n">
         <v>47721</v>
       </c>
-      <c r="G49" s="95">
+      <c r="G49" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -44044,7 +44082,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I49" s="96" t="n">
+      <c r="I49" s="98" t="n">
         <v>170732.54</v>
       </c>
       <c r="J49" s="26" t="n">
@@ -44087,7 +44125,7 @@
       <c r="F50" s="91" t="n">
         <v>47721</v>
       </c>
-      <c r="G50" s="95">
+      <c r="G50" s="97">
         <f>tblAuftraege[[#This Row],[Einnahmen]]/1.299</f>
         <v/>
       </c>
@@ -44096,7 +44134,7 @@
 Ausgaben]]+112</f>
         <v/>
       </c>
-      <c r="I50" s="96" t="n">
+      <c r="I50" s="98" t="n">
         <v>66447.57000000001</v>
       </c>
       <c r="J50" s="26" t="n">
@@ -44139,14 +44177,14 @@
       <c r="F51" s="28" t="n">
         <v>46402</v>
       </c>
-      <c r="G51" s="95">
+      <c r="G51" s="97">
         <f>1115.5+46560</f>
         <v/>
       </c>
       <c r="H51" s="24" t="n">
         <v>46440</v>
       </c>
-      <c r="I51" s="96" t="n">
+      <c r="I51" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J51" s="26" t="n">
@@ -44191,13 +44229,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G52" s="95" t="n">
+      <c r="G52" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H52" s="24" t="n">
         <v>46517</v>
       </c>
-      <c r="I52" s="96" t="n">
+      <c r="I52" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J52" s="26" t="n">
@@ -44242,13 +44280,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G53" s="95" t="n">
+      <c r="G53" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H53" s="24" t="n">
         <v>46608</v>
       </c>
-      <c r="I53" s="96" t="n">
+      <c r="I53" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J53" s="26" t="n">
@@ -44293,13 +44331,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G54" s="95" t="n">
+      <c r="G54" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H54" s="24" t="n">
         <v>46622</v>
       </c>
-      <c r="I54" s="96" t="n">
+      <c r="I54" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J54" s="26" t="n">
@@ -44344,13 +44382,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G55" s="95" t="n">
+      <c r="G55" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H55" s="24" t="n">
         <v>46650</v>
       </c>
-      <c r="I55" s="96" t="n">
+      <c r="I55" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J55" s="26" t="n">
@@ -44395,13 +44433,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G56" s="95" t="n">
+      <c r="G56" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H56" s="24" t="n">
         <v>46664</v>
       </c>
-      <c r="I56" s="96" t="n">
+      <c r="I56" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J56" s="26" t="n">
@@ -44446,13 +44484,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G57" s="95" t="n">
+      <c r="G57" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H57" s="24" t="n">
         <v>46797</v>
       </c>
-      <c r="I57" s="96" t="n">
+      <c r="I57" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J57" s="26" t="n">
@@ -44497,13 +44535,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G58" s="95" t="n">
+      <c r="G58" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H58" s="24" t="n">
         <v>46811</v>
       </c>
-      <c r="I58" s="96" t="n">
+      <c r="I58" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J58" s="26" t="n">
@@ -44548,13 +44586,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G59" s="95" t="n">
+      <c r="G59" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H59" s="24" t="n">
         <v>46818</v>
       </c>
-      <c r="I59" s="96" t="n">
+      <c r="I59" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J59" s="26" t="n">
@@ -44599,13 +44637,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G60" s="95" t="n">
+      <c r="G60" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H60" s="24" t="n">
         <v>46881</v>
       </c>
-      <c r="I60" s="96" t="n">
+      <c r="I60" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J60" s="26" t="n">
@@ -44650,13 +44688,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G61" s="95" t="n">
+      <c r="G61" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H61" s="24" t="n">
         <v>46888</v>
       </c>
-      <c r="I61" s="96" t="n">
+      <c r="I61" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J61" s="26" t="n">
@@ -44701,13 +44739,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G62" s="95" t="n">
+      <c r="G62" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H62" s="24" t="n">
         <v>47126</v>
       </c>
-      <c r="I62" s="96" t="n">
+      <c r="I62" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J62" s="26" t="n">
@@ -44752,13 +44790,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G63" s="95" t="n">
+      <c r="G63" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H63" s="24" t="n">
         <v>47196</v>
       </c>
-      <c r="I63" s="96" t="n">
+      <c r="I63" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J63" s="26" t="n">
@@ -44803,13 +44841,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G64" s="95" t="n">
+      <c r="G64" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H64" s="24" t="n">
         <v>47315</v>
       </c>
-      <c r="I64" s="96" t="n">
+      <c r="I64" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J64" s="26" t="n">
@@ -44854,13 +44892,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G65" s="95" t="n">
+      <c r="G65" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H65" s="24" t="n">
         <v>47196</v>
       </c>
-      <c r="I65" s="96" t="n">
+      <c r="I65" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J65" s="26" t="n">
@@ -44905,13 +44943,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G66" s="95" t="n">
+      <c r="G66" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H66" s="24" t="n">
         <v>47357</v>
       </c>
-      <c r="I66" s="96" t="n">
+      <c r="I66" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J66" s="26" t="n">
@@ -44956,13 +44994,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G67" s="95" t="n">
+      <c r="G67" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H67" s="24" t="n">
         <v>47546</v>
       </c>
-      <c r="I67" s="96" t="n">
+      <c r="I67" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J67" s="26" t="n">
@@ -45007,13 +45045,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G68" s="95" t="n">
+      <c r="G68" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H68" s="24" t="n">
         <v>47546</v>
       </c>
-      <c r="I68" s="96" t="n">
+      <c r="I68" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J68" s="26" t="n">
@@ -45058,13 +45096,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G69" s="95" t="n">
+      <c r="G69" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H69" s="24" t="n">
         <v>47567</v>
       </c>
-      <c r="I69" s="96" t="n">
+      <c r="I69" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J69" s="26" t="n">
@@ -45109,13 +45147,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G70" s="95" t="n">
+      <c r="G70" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H70" s="24" t="n">
         <v>47588</v>
       </c>
-      <c r="I70" s="96" t="n">
+      <c r="I70" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J70" s="26" t="n">
@@ -45160,13 +45198,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G71" s="95" t="n">
+      <c r="G71" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H71" s="24" t="n">
         <v>47588</v>
       </c>
-      <c r="I71" s="96" t="n">
+      <c r="I71" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J71" s="26" t="n">
@@ -45211,13 +45249,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G72" s="95" t="n">
+      <c r="G72" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H72" s="24" t="n">
         <v>47588</v>
       </c>
-      <c r="I72" s="96" t="n">
+      <c r="I72" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J72" s="26" t="n">
@@ -45262,13 +45300,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G73" s="95" t="n">
+      <c r="G73" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H73" s="24" t="n">
         <v>47721</v>
       </c>
-      <c r="I73" s="96" t="n">
+      <c r="I73" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J73" s="26" t="n">
@@ -45313,13 +45351,13 @@
 Einnahmen]]-84</f>
         <v/>
       </c>
-      <c r="G74" s="95" t="n">
+      <c r="G74" s="97" t="n">
         <v>1115.5</v>
       </c>
       <c r="H74" s="24" t="n">
         <v>47721</v>
       </c>
-      <c r="I74" s="96" t="n">
+      <c r="I74" s="98" t="n">
         <v>11267.28</v>
       </c>
       <c r="J74" s="26" t="n">
@@ -45362,13 +45400,13 @@
       <c r="F75" s="28" t="n">
         <v>46522</v>
       </c>
-      <c r="G75" s="95" t="n">
+      <c r="G75" s="97" t="n">
         <v>3750</v>
       </c>
       <c r="H75" s="24" t="n">
         <v>46583</v>
       </c>
-      <c r="I75" s="96">
+      <c r="I75" s="98">
         <f>1748.52*3</f>
         <v/>
       </c>
@@ -45410,9 +45448,9 @@
         </is>
       </c>
       <c r="F76" s="28" t="n"/>
-      <c r="G76" s="95" t="n"/>
+      <c r="G76" s="97" t="n"/>
       <c r="H76" s="24" t="n"/>
-      <c r="I76" s="96" t="n"/>
+      <c r="I76" s="98" t="n"/>
       <c r="J76" s="26" t="n">
         <v>1</v>
       </c>
@@ -45451,9 +45489,9 @@
         </is>
       </c>
       <c r="F77" s="28" t="n"/>
-      <c r="G77" s="95" t="n"/>
+      <c r="G77" s="97" t="n"/>
       <c r="H77" s="24" t="n"/>
-      <c r="I77" s="96" t="n"/>
+      <c r="I77" s="98" t="n"/>
       <c r="J77" s="26" t="n">
         <v>1</v>
       </c>
@@ -45492,9 +45530,9 @@
         </is>
       </c>
       <c r="F78" s="28" t="n"/>
-      <c r="G78" s="95" t="n"/>
+      <c r="G78" s="97" t="n"/>
       <c r="H78" s="24" t="n"/>
-      <c r="I78" s="96" t="n"/>
+      <c r="I78" s="98" t="n"/>
       <c r="J78" s="26" t="n">
         <v>1</v>
       </c>
@@ -45533,9 +45571,9 @@
         </is>
       </c>
       <c r="F79" s="28" t="n"/>
-      <c r="G79" s="95" t="n"/>
+      <c r="G79" s="97" t="n"/>
       <c r="H79" s="24" t="n"/>
-      <c r="I79" s="96" t="n"/>
+      <c r="I79" s="98" t="n"/>
       <c r="J79" s="26" t="n">
         <v>1</v>
       </c>
@@ -45574,9 +45612,9 @@
         </is>
       </c>
       <c r="F80" s="28" t="n"/>
-      <c r="G80" s="95" t="n"/>
+      <c r="G80" s="97" t="n"/>
       <c r="H80" s="24" t="n"/>
-      <c r="I80" s="96" t="n"/>
+      <c r="I80" s="98" t="n"/>
       <c r="J80" s="26" t="n">
         <v>1</v>
       </c>
@@ -45615,9 +45653,9 @@
         </is>
       </c>
       <c r="F81" s="28" t="n"/>
-      <c r="G81" s="95" t="n"/>
+      <c r="G81" s="97" t="n"/>
       <c r="H81" s="24" t="n"/>
-      <c r="I81" s="96" t="n"/>
+      <c r="I81" s="98" t="n"/>
       <c r="J81" s="26" t="n">
         <v>1</v>
       </c>
@@ -45656,9 +45694,9 @@
         </is>
       </c>
       <c r="F82" s="28" t="n"/>
-      <c r="G82" s="95" t="n"/>
+      <c r="G82" s="97" t="n"/>
       <c r="H82" s="24" t="n"/>
-      <c r="I82" s="96" t="n"/>
+      <c r="I82" s="98" t="n"/>
       <c r="J82" s="26" t="n">
         <v>1</v>
       </c>
@@ -45697,9 +45735,9 @@
         </is>
       </c>
       <c r="F83" s="28" t="n"/>
-      <c r="G83" s="95" t="n"/>
+      <c r="G83" s="97" t="n"/>
       <c r="H83" s="24" t="n"/>
-      <c r="I83" s="96" t="n"/>
+      <c r="I83" s="98" t="n"/>
       <c r="J83" s="26" t="n">
         <v>1</v>
       </c>
@@ -45738,9 +45776,9 @@
         </is>
       </c>
       <c r="F84" s="28" t="n"/>
-      <c r="G84" s="95" t="n"/>
+      <c r="G84" s="97" t="n"/>
       <c r="H84" s="24" t="n"/>
-      <c r="I84" s="96" t="n"/>
+      <c r="I84" s="98" t="n"/>
       <c r="J84" s="26" t="n">
         <v>1</v>
       </c>
@@ -45779,9 +45817,9 @@
         </is>
       </c>
       <c r="F85" s="28" t="n"/>
-      <c r="G85" s="95" t="n"/>
+      <c r="G85" s="97" t="n"/>
       <c r="H85" s="24" t="n"/>
-      <c r="I85" s="96" t="n"/>
+      <c r="I85" s="98" t="n"/>
       <c r="J85" s="26" t="n">
         <v>1</v>
       </c>
@@ -45820,9 +45858,9 @@
         </is>
       </c>
       <c r="F86" s="28" t="n"/>
-      <c r="G86" s="95" t="n"/>
+      <c r="G86" s="97" t="n"/>
       <c r="H86" s="24" t="n"/>
-      <c r="I86" s="96" t="n"/>
+      <c r="I86" s="98" t="n"/>
       <c r="J86" s="26" t="n">
         <v>1</v>
       </c>
@@ -45861,9 +45899,9 @@
         </is>
       </c>
       <c r="F87" s="28" t="n"/>
-      <c r="G87" s="95" t="n"/>
+      <c r="G87" s="97" t="n"/>
       <c r="H87" s="24" t="n"/>
-      <c r="I87" s="96" t="n"/>
+      <c r="I87" s="98" t="n"/>
       <c r="J87" s="26" t="n">
         <v>1</v>
       </c>
@@ -45902,9 +45940,9 @@
         </is>
       </c>
       <c r="F88" s="28" t="n"/>
-      <c r="G88" s="95" t="n"/>
+      <c r="G88" s="97" t="n"/>
       <c r="H88" s="24" t="n"/>
-      <c r="I88" s="96" t="n"/>
+      <c r="I88" s="98" t="n"/>
       <c r="J88" s="26" t="n">
         <v>1</v>
       </c>
@@ -45943,9 +45981,9 @@
         </is>
       </c>
       <c r="F89" s="28" t="n"/>
-      <c r="G89" s="95" t="n"/>
+      <c r="G89" s="97" t="n"/>
       <c r="H89" s="24" t="n"/>
-      <c r="I89" s="96" t="n"/>
+      <c r="I89" s="98" t="n"/>
       <c r="J89" s="26" t="n">
         <v>1</v>
       </c>
@@ -45984,9 +46022,9 @@
         </is>
       </c>
       <c r="F90" s="28" t="n"/>
-      <c r="G90" s="95" t="n"/>
+      <c r="G90" s="97" t="n"/>
       <c r="H90" s="24" t="n"/>
-      <c r="I90" s="96" t="n"/>
+      <c r="I90" s="98" t="n"/>
       <c r="J90" s="26" t="n">
         <v>1</v>
       </c>
@@ -46025,9 +46063,9 @@
         </is>
       </c>
       <c r="F91" s="28" t="n"/>
-      <c r="G91" s="95" t="n"/>
+      <c r="G91" s="97" t="n"/>
       <c r="H91" s="24" t="n"/>
-      <c r="I91" s="96" t="n"/>
+      <c r="I91" s="98" t="n"/>
       <c r="J91" s="26" t="n">
         <v>1</v>
       </c>
@@ -46066,9 +46104,9 @@
         </is>
       </c>
       <c r="F92" s="28" t="n"/>
-      <c r="G92" s="95" t="n"/>
+      <c r="G92" s="97" t="n"/>
       <c r="H92" s="24" t="n"/>
-      <c r="I92" s="96" t="n"/>
+      <c r="I92" s="98" t="n"/>
       <c r="J92" s="26" t="n">
         <v>1</v>
       </c>
@@ -46107,9 +46145,9 @@
         </is>
       </c>
       <c r="F93" s="28" t="n"/>
-      <c r="G93" s="95" t="n"/>
+      <c r="G93" s="97" t="n"/>
       <c r="H93" s="24" t="n"/>
-      <c r="I93" s="96" t="n"/>
+      <c r="I93" s="98" t="n"/>
       <c r="J93" s="26" t="n">
         <v>1</v>
       </c>
@@ -46148,9 +46186,9 @@
         </is>
       </c>
       <c r="F94" s="28" t="n"/>
-      <c r="G94" s="95" t="n"/>
+      <c r="G94" s="97" t="n"/>
       <c r="H94" s="24" t="n"/>
-      <c r="I94" s="96" t="n"/>
+      <c r="I94" s="98" t="n"/>
       <c r="J94" s="26" t="n">
         <v>1</v>
       </c>
@@ -46189,9 +46227,9 @@
         </is>
       </c>
       <c r="F95" s="28" t="n"/>
-      <c r="G95" s="95" t="n"/>
+      <c r="G95" s="97" t="n"/>
       <c r="H95" s="24" t="n"/>
-      <c r="I95" s="96" t="n"/>
+      <c r="I95" s="98" t="n"/>
       <c r="J95" s="26" t="n">
         <v>1</v>
       </c>
@@ -46230,9 +46268,9 @@
         </is>
       </c>
       <c r="F96" s="28" t="n"/>
-      <c r="G96" s="95" t="n"/>
+      <c r="G96" s="97" t="n"/>
       <c r="H96" s="24" t="n"/>
-      <c r="I96" s="96" t="n"/>
+      <c r="I96" s="98" t="n"/>
       <c r="J96" s="26" t="n">
         <v>1</v>
       </c>
@@ -46271,9 +46309,9 @@
         </is>
       </c>
       <c r="F97" s="28" t="n"/>
-      <c r="G97" s="95" t="n"/>
+      <c r="G97" s="97" t="n"/>
       <c r="H97" s="24" t="n"/>
-      <c r="I97" s="96" t="n"/>
+      <c r="I97" s="98" t="n"/>
       <c r="J97" s="26" t="n">
         <v>1</v>
       </c>
@@ -46312,9 +46350,9 @@
         </is>
       </c>
       <c r="F98" s="28" t="n"/>
-      <c r="G98" s="95" t="n"/>
+      <c r="G98" s="97" t="n"/>
       <c r="H98" s="24" t="n"/>
-      <c r="I98" s="96" t="n"/>
+      <c r="I98" s="98" t="n"/>
       <c r="J98" s="26" t="n">
         <v>1</v>
       </c>
@@ -46355,11 +46393,11 @@
       <c r="F99" s="28" t="n">
         <v>46249</v>
       </c>
-      <c r="G99" s="95" t="n"/>
+      <c r="G99" s="97" t="n"/>
       <c r="H99" s="24" t="n">
         <v>46326</v>
       </c>
-      <c r="I99" s="96" t="n">
+      <c r="I99" s="98" t="n">
         <v>3200</v>
       </c>
       <c r="J99" s="26" t="n">
@@ -46402,11 +46440,11 @@
       <c r="F100" s="28" t="n">
         <v>46249</v>
       </c>
-      <c r="G100" s="95" t="n"/>
+      <c r="G100" s="97" t="n"/>
       <c r="H100" s="24" t="n">
         <v>46310</v>
       </c>
-      <c r="I100" s="96" t="n"/>
+      <c r="I100" s="98" t="n"/>
       <c r="J100" s="26" t="n">
         <v>1</v>
       </c>
@@ -46447,11 +46485,11 @@
       <c r="F101" s="28" t="n">
         <v>46341</v>
       </c>
-      <c r="G101" s="95" t="n"/>
+      <c r="G101" s="97" t="n"/>
       <c r="H101" s="24" t="n">
         <v>46402</v>
       </c>
-      <c r="I101" s="96" t="n"/>
+      <c r="I101" s="98" t="n"/>
       <c r="J101" s="26" t="n">
         <v>1</v>
       </c>
@@ -46492,11 +46530,11 @@
       <c r="F102" s="28" t="n">
         <v>46433</v>
       </c>
-      <c r="G102" s="95" t="n"/>
+      <c r="G102" s="97" t="n"/>
       <c r="H102" s="24" t="n">
         <v>46492</v>
       </c>
-      <c r="I102" s="96" t="n"/>
+      <c r="I102" s="98" t="n"/>
       <c r="J102" s="26" t="n">
         <v>1</v>
       </c>
@@ -46537,11 +46575,11 @@
       <c r="F103" s="28" t="n">
         <v>46522</v>
       </c>
-      <c r="G103" s="95" t="n"/>
+      <c r="G103" s="97" t="n"/>
       <c r="H103" s="24" t="n">
         <v>46583</v>
       </c>
-      <c r="I103" s="96" t="n"/>
+      <c r="I103" s="98" t="n"/>
       <c r="J103" s="26" t="n">
         <v>1</v>
       </c>
@@ -46582,11 +46620,11 @@
       <c r="F104" s="28" t="n">
         <v>46614</v>
       </c>
-      <c r="G104" s="95" t="n"/>
+      <c r="G104" s="97" t="n"/>
       <c r="H104" s="24" t="n">
         <v>46675</v>
       </c>
-      <c r="I104" s="96" t="n"/>
+      <c r="I104" s="98" t="n"/>
       <c r="J104" s="26" t="n">
         <v>1</v>
       </c>
@@ -46627,13 +46665,13 @@
       <c r="F105" s="28" t="n">
         <v>46706</v>
       </c>
-      <c r="G105" s="95" t="n">
+      <c r="G105" s="97" t="n">
         <v>10000</v>
       </c>
       <c r="H105" s="24" t="n">
         <v>46767</v>
       </c>
-      <c r="I105" s="96" t="n">
+      <c r="I105" s="98" t="n">
         <v>13000</v>
       </c>
       <c r="J105" s="26" t="n">
@@ -46680,11 +46718,11 @@
       <c r="F106" s="28" t="n">
         <v>46037</v>
       </c>
-      <c r="G106" s="98" t="n">
+      <c r="G106" s="100" t="n">
         <v>12000</v>
       </c>
       <c r="H106" s="24" t="n"/>
-      <c r="I106" s="96" t="n"/>
+      <c r="I106" s="98" t="n"/>
       <c r="J106" s="26" t="n">
         <v>1</v>
       </c>
@@ -46725,13 +46763,13 @@
       <c r="F107" s="28" t="n">
         <v>46282</v>
       </c>
-      <c r="G107" s="95" t="n">
+      <c r="G107" s="97" t="n">
         <v>4741.26</v>
       </c>
       <c r="H107" s="24" t="n">
         <v>46309</v>
       </c>
-      <c r="I107" s="96" t="n">
+      <c r="I107" s="98" t="n">
         <v>8421.02</v>
       </c>
       <c r="J107" s="26" t="n">
@@ -46778,13 +46816,13 @@
       <c r="F108" s="28" t="n">
         <v>46274</v>
       </c>
-      <c r="G108" s="95" t="n">
+      <c r="G108" s="97" t="n">
         <v>1985.06</v>
       </c>
       <c r="H108" s="24" t="n">
         <v>46307</v>
       </c>
-      <c r="I108" s="96" t="n">
+      <c r="I108" s="98" t="n">
         <v>3441.4</v>
       </c>
       <c r="J108" s="26" t="n">
@@ -46827,11 +46865,11 @@
       <c r="F109" s="28" t="n">
         <v>46276</v>
       </c>
-      <c r="G109" s="95" t="n"/>
+      <c r="G109" s="97" t="n"/>
       <c r="H109" s="24" t="n">
         <v>46279</v>
       </c>
-      <c r="I109" s="96" t="n">
+      <c r="I109" s="98" t="n">
         <v>2480</v>
       </c>
       <c r="J109" s="26" t="n">
@@ -46878,13 +46916,13 @@
       <c r="F110" s="28" t="n">
         <v>46371</v>
       </c>
-      <c r="G110" s="95" t="n">
+      <c r="G110" s="97" t="n">
         <v>10000</v>
       </c>
       <c r="H110" s="24" t="n">
         <v>46371</v>
       </c>
-      <c r="I110" s="96" t="n">
+      <c r="I110" s="98" t="n">
         <v>16500</v>
       </c>
       <c r="J110" s="26" t="n">
@@ -46931,13 +46969,13 @@
       <c r="F111" s="28" t="n">
         <v>46232</v>
       </c>
-      <c r="G111" s="95" t="n">
+      <c r="G111" s="97" t="n">
         <v>924.88</v>
       </c>
       <c r="H111" s="24" t="n">
         <v>46261</v>
       </c>
-      <c r="I111" s="96" t="n">
+      <c r="I111" s="98" t="n">
         <v>1745.6</v>
       </c>
       <c r="J111" s="26" t="n">
@@ -46980,13 +47018,13 @@
       <c r="F112" s="28" t="n">
         <v>46310</v>
       </c>
-      <c r="G112" s="95" t="n">
+      <c r="G112" s="97" t="n">
         <v>132405.13</v>
       </c>
       <c r="H112" s="24" t="n">
         <v>46371</v>
       </c>
-      <c r="I112" s="96" t="n">
+      <c r="I112" s="98" t="n">
         <v>169319.25</v>
       </c>
       <c r="J112" s="26" t="n">
@@ -47027,9 +47065,9 @@
         </is>
       </c>
       <c r="F113" s="28" t="n"/>
-      <c r="G113" s="95" t="n"/>
+      <c r="G113" s="97" t="n"/>
       <c r="H113" s="24" t="n"/>
-      <c r="I113" s="96" t="n">
+      <c r="I113" s="98" t="n">
         <v>3864.18</v>
       </c>
       <c r="J113" s="26" t="n">
@@ -47072,11 +47110,11 @@
       <c r="F114" s="28" t="n">
         <v>46272</v>
       </c>
-      <c r="G114" s="95" t="n"/>
+      <c r="G114" s="97" t="n"/>
       <c r="H114" s="24" t="n">
         <v>46298</v>
       </c>
-      <c r="I114" s="96" t="n">
+      <c r="I114" s="98" t="n">
         <v>8050</v>
       </c>
       <c r="J114" s="26" t="n">
@@ -47105,9 +47143,9 @@
       <c r="D115" s="22" t="n"/>
       <c r="E115" s="22" t="n"/>
       <c r="F115" s="28" t="n"/>
-      <c r="G115" s="95" t="n"/>
+      <c r="G115" s="97" t="n"/>
       <c r="H115" s="24" t="n"/>
-      <c r="I115" s="96" t="n"/>
+      <c r="I115" s="98" t="n"/>
       <c r="J115" s="26" t="n">
         <v>1</v>
       </c>
@@ -47130,9 +47168,9 @@
       <c r="D116" s="22" t="n"/>
       <c r="E116" s="22" t="n"/>
       <c r="F116" s="28" t="n"/>
-      <c r="G116" s="95" t="n"/>
+      <c r="G116" s="97" t="n"/>
       <c r="H116" s="24" t="n"/>
-      <c r="I116" s="96" t="n"/>
+      <c r="I116" s="98" t="n"/>
       <c r="J116" s="26" t="n">
         <v>1</v>
       </c>
@@ -47155,9 +47193,9 @@
       <c r="D117" s="22" t="n"/>
       <c r="E117" s="22" t="n"/>
       <c r="F117" s="28" t="n"/>
-      <c r="G117" s="95" t="n"/>
+      <c r="G117" s="97" t="n"/>
       <c r="H117" s="24" t="n"/>
-      <c r="I117" s="96" t="n"/>
+      <c r="I117" s="98" t="n"/>
       <c r="J117" s="26" t="n">
         <v>1</v>
       </c>
@@ -47180,9 +47218,9 @@
       <c r="D118" s="22" t="n"/>
       <c r="E118" s="22" t="n"/>
       <c r="F118" s="28" t="n"/>
-      <c r="G118" s="95" t="n"/>
+      <c r="G118" s="97" t="n"/>
       <c r="H118" s="24" t="n"/>
-      <c r="I118" s="96" t="n"/>
+      <c r="I118" s="98" t="n"/>
       <c r="J118" s="26" t="n">
         <v>1</v>
       </c>
@@ -47205,9 +47243,9 @@
       <c r="D119" s="22" t="n"/>
       <c r="E119" s="22" t="n"/>
       <c r="F119" s="28" t="n"/>
-      <c r="G119" s="95" t="n"/>
+      <c r="G119" s="97" t="n"/>
       <c r="H119" s="24" t="n"/>
-      <c r="I119" s="96" t="n"/>
+      <c r="I119" s="98" t="n"/>
       <c r="J119" s="26" t="n">
         <v>1</v>
       </c>
@@ -47230,9 +47268,9 @@
       <c r="D120" s="22" t="n"/>
       <c r="E120" s="22" t="n"/>
       <c r="F120" s="28" t="n"/>
-      <c r="G120" s="95" t="n"/>
+      <c r="G120" s="97" t="n"/>
       <c r="H120" s="24" t="n"/>
-      <c r="I120" s="96" t="n"/>
+      <c r="I120" s="98" t="n"/>
       <c r="J120" s="26" t="n">
         <v>1</v>
       </c>
@@ -47255,9 +47293,9 @@
       <c r="D121" s="22" t="n"/>
       <c r="E121" s="22" t="n"/>
       <c r="F121" s="28" t="n"/>
-      <c r="G121" s="95" t="n"/>
+      <c r="G121" s="97" t="n"/>
       <c r="H121" s="24" t="n"/>
-      <c r="I121" s="96" t="n"/>
+      <c r="I121" s="98" t="n"/>
       <c r="J121" s="26" t="n">
         <v>1</v>
       </c>
@@ -47280,9 +47318,9 @@
       <c r="D122" s="22" t="n"/>
       <c r="E122" s="22" t="n"/>
       <c r="F122" s="28" t="n"/>
-      <c r="G122" s="95" t="n"/>
+      <c r="G122" s="97" t="n"/>
       <c r="H122" s="24" t="n"/>
-      <c r="I122" s="96" t="n"/>
+      <c r="I122" s="98" t="n"/>
       <c r="J122" s="26" t="n">
         <v>1</v>
       </c>
@@ -47305,9 +47343,9 @@
       <c r="D123" s="22" t="n"/>
       <c r="E123" s="22" t="n"/>
       <c r="F123" s="28" t="n"/>
-      <c r="G123" s="95" t="n"/>
+      <c r="G123" s="97" t="n"/>
       <c r="H123" s="24" t="n"/>
-      <c r="I123" s="96" t="n"/>
+      <c r="I123" s="98" t="n"/>
       <c r="J123" s="26" t="n">
         <v>1</v>
       </c>
@@ -47330,9 +47368,9 @@
       <c r="D124" s="22" t="n"/>
       <c r="E124" s="22" t="n"/>
       <c r="F124" s="28" t="n"/>
-      <c r="G124" s="95" t="n"/>
+      <c r="G124" s="97" t="n"/>
       <c r="H124" s="24" t="n"/>
-      <c r="I124" s="96" t="n"/>
+      <c r="I124" s="98" t="n"/>
       <c r="J124" s="26" t="n">
         <v>1</v>
       </c>
@@ -47355,9 +47393,9 @@
       <c r="D125" s="22" t="n"/>
       <c r="E125" s="22" t="n"/>
       <c r="F125" s="28" t="n"/>
-      <c r="G125" s="95" t="n"/>
+      <c r="G125" s="97" t="n"/>
       <c r="H125" s="24" t="n"/>
-      <c r="I125" s="96" t="n"/>
+      <c r="I125" s="98" t="n"/>
       <c r="J125" s="26" t="n">
         <v>1</v>
       </c>
@@ -47380,9 +47418,9 @@
       <c r="D126" s="22" t="n"/>
       <c r="E126" s="22" t="n"/>
       <c r="F126" s="28" t="n"/>
-      <c r="G126" s="95" t="n"/>
+      <c r="G126" s="97" t="n"/>
       <c r="H126" s="24" t="n"/>
-      <c r="I126" s="96" t="n"/>
+      <c r="I126" s="98" t="n"/>
       <c r="J126" s="26" t="n">
         <v>1</v>
       </c>
@@ -47405,9 +47443,9 @@
       <c r="D127" s="22" t="n"/>
       <c r="E127" s="22" t="n"/>
       <c r="F127" s="28" t="n"/>
-      <c r="G127" s="95" t="n"/>
+      <c r="G127" s="97" t="n"/>
       <c r="H127" s="24" t="n"/>
-      <c r="I127" s="96" t="n"/>
+      <c r="I127" s="98" t="n"/>
       <c r="J127" s="26" t="n">
         <v>1</v>
       </c>
@@ -47430,9 +47468,9 @@
       <c r="D128" s="22" t="n"/>
       <c r="E128" s="22" t="n"/>
       <c r="F128" s="28" t="n"/>
-      <c r="G128" s="95" t="n"/>
+      <c r="G128" s="97" t="n"/>
       <c r="H128" s="24" t="n"/>
-      <c r="I128" s="96" t="n"/>
+      <c r="I128" s="98" t="n"/>
       <c r="J128" s="26" t="n">
         <v>1</v>
       </c>
@@ -47455,9 +47493,9 @@
       <c r="D129" s="22" t="n"/>
       <c r="E129" s="22" t="n"/>
       <c r="F129" s="28" t="n"/>
-      <c r="G129" s="95" t="n"/>
+      <c r="G129" s="97" t="n"/>
       <c r="H129" s="24" t="n"/>
-      <c r="I129" s="96" t="n"/>
+      <c r="I129" s="98" t="n"/>
       <c r="J129" s="26" t="n">
         <v>1</v>
       </c>
@@ -47480,9 +47518,9 @@
       <c r="D130" s="22" t="n"/>
       <c r="E130" s="22" t="n"/>
       <c r="F130" s="28" t="n"/>
-      <c r="G130" s="95" t="n"/>
+      <c r="G130" s="97" t="n"/>
       <c r="H130" s="24" t="n"/>
-      <c r="I130" s="96" t="n"/>
+      <c r="I130" s="98" t="n"/>
       <c r="J130" s="26" t="n">
         <v>1</v>
       </c>
@@ -47505,9 +47543,9 @@
       <c r="D131" s="22" t="n"/>
       <c r="E131" s="22" t="n"/>
       <c r="F131" s="28" t="n"/>
-      <c r="G131" s="95" t="n"/>
+      <c r="G131" s="97" t="n"/>
       <c r="H131" s="24" t="n"/>
-      <c r="I131" s="96" t="n"/>
+      <c r="I131" s="98" t="n"/>
       <c r="J131" s="26" t="n">
         <v>1</v>
       </c>
@@ -47530,9 +47568,9 @@
       <c r="D132" s="22" t="n"/>
       <c r="E132" s="22" t="n"/>
       <c r="F132" s="28" t="n"/>
-      <c r="G132" s="95" t="n"/>
+      <c r="G132" s="97" t="n"/>
       <c r="H132" s="24" t="n"/>
-      <c r="I132" s="96" t="n"/>
+      <c r="I132" s="98" t="n"/>
       <c r="J132" s="26" t="n">
         <v>1</v>
       </c>
@@ -47555,9 +47593,9 @@
       <c r="D133" s="22" t="n"/>
       <c r="E133" s="22" t="n"/>
       <c r="F133" s="28" t="n"/>
-      <c r="G133" s="95" t="n"/>
+      <c r="G133" s="97" t="n"/>
       <c r="H133" s="24" t="n"/>
-      <c r="I133" s="96" t="n"/>
+      <c r="I133" s="98" t="n"/>
       <c r="J133" s="26" t="n">
         <v>1</v>
       </c>
@@ -47580,9 +47618,9 @@
       <c r="D134" s="22" t="n"/>
       <c r="E134" s="22" t="n"/>
       <c r="F134" s="28" t="n"/>
-      <c r="G134" s="95" t="n"/>
+      <c r="G134" s="97" t="n"/>
       <c r="H134" s="24" t="n"/>
-      <c r="I134" s="96" t="n"/>
+      <c r="I134" s="98" t="n"/>
       <c r="J134" s="26" t="n">
         <v>1</v>
       </c>
@@ -47605,9 +47643,9 @@
       <c r="D135" s="22" t="n"/>
       <c r="E135" s="22" t="n"/>
       <c r="F135" s="28" t="n"/>
-      <c r="G135" s="95" t="n"/>
+      <c r="G135" s="97" t="n"/>
       <c r="H135" s="24" t="n"/>
-      <c r="I135" s="96" t="n"/>
+      <c r="I135" s="98" t="n"/>
       <c r="J135" s="26" t="n">
         <v>1</v>
       </c>
@@ -47630,9 +47668,9 @@
       <c r="D136" s="22" t="n"/>
       <c r="E136" s="22" t="n"/>
       <c r="F136" s="28" t="n"/>
-      <c r="G136" s="95" t="n"/>
+      <c r="G136" s="97" t="n"/>
       <c r="H136" s="24" t="n"/>
-      <c r="I136" s="96" t="n"/>
+      <c r="I136" s="98" t="n"/>
       <c r="J136" s="26" t="n">
         <v>1</v>
       </c>
@@ -47655,9 +47693,9 @@
       <c r="D137" s="22" t="n"/>
       <c r="E137" s="22" t="n"/>
       <c r="F137" s="28" t="n"/>
-      <c r="G137" s="95" t="n"/>
+      <c r="G137" s="97" t="n"/>
       <c r="H137" s="24" t="n"/>
-      <c r="I137" s="96" t="n"/>
+      <c r="I137" s="98" t="n"/>
       <c r="J137" s="26" t="n">
         <v>1</v>
       </c>
@@ -47680,9 +47718,9 @@
       <c r="D138" s="22" t="n"/>
       <c r="E138" s="22" t="n"/>
       <c r="F138" s="28" t="n"/>
-      <c r="G138" s="95" t="n"/>
+      <c r="G138" s="97" t="n"/>
       <c r="H138" s="24" t="n"/>
-      <c r="I138" s="96" t="n"/>
+      <c r="I138" s="98" t="n"/>
       <c r="J138" s="26" t="n">
         <v>1</v>
       </c>
@@ -47705,9 +47743,9 @@
       <c r="D139" s="22" t="n"/>
       <c r="E139" s="22" t="n"/>
       <c r="F139" s="28" t="n"/>
-      <c r="G139" s="95" t="n"/>
+      <c r="G139" s="97" t="n"/>
       <c r="H139" s="24" t="n"/>
-      <c r="I139" s="96" t="n"/>
+      <c r="I139" s="98" t="n"/>
       <c r="J139" s="26" t="n">
         <v>1</v>
       </c>
@@ -47730,9 +47768,9 @@
       <c r="D140" s="22" t="n"/>
       <c r="E140" s="22" t="n"/>
       <c r="F140" s="28" t="n"/>
-      <c r="G140" s="95" t="n"/>
+      <c r="G140" s="97" t="n"/>
       <c r="H140" s="24" t="n"/>
-      <c r="I140" s="96" t="n"/>
+      <c r="I140" s="98" t="n"/>
       <c r="J140" s="26" t="n">
         <v>1</v>
       </c>
@@ -47755,9 +47793,9 @@
       <c r="D141" s="22" t="n"/>
       <c r="E141" s="22" t="n"/>
       <c r="F141" s="28" t="n"/>
-      <c r="G141" s="95" t="n"/>
+      <c r="G141" s="97" t="n"/>
       <c r="H141" s="24" t="n"/>
-      <c r="I141" s="96" t="n"/>
+      <c r="I141" s="98" t="n"/>
       <c r="J141" s="26" t="n">
         <v>1</v>
       </c>
@@ -47780,9 +47818,9 @@
       <c r="D142" s="22" t="n"/>
       <c r="E142" s="22" t="n"/>
       <c r="F142" s="28" t="n"/>
-      <c r="G142" s="95" t="n"/>
+      <c r="G142" s="97" t="n"/>
       <c r="H142" s="24" t="n"/>
-      <c r="I142" s="96" t="n"/>
+      <c r="I142" s="98" t="n"/>
       <c r="J142" s="26" t="n">
         <v>1</v>
       </c>
@@ -47805,9 +47843,9 @@
       <c r="D143" s="22" t="n"/>
       <c r="E143" s="22" t="n"/>
       <c r="F143" s="28" t="n"/>
-      <c r="G143" s="95" t="n"/>
+      <c r="G143" s="97" t="n"/>
       <c r="H143" s="24" t="n"/>
-      <c r="I143" s="96" t="n"/>
+      <c r="I143" s="98" t="n"/>
       <c r="J143" s="26" t="n">
         <v>1</v>
       </c>
@@ -47830,9 +47868,9 @@
       <c r="D144" s="22" t="n"/>
       <c r="E144" s="22" t="n"/>
       <c r="F144" s="28" t="n"/>
-      <c r="G144" s="95" t="n"/>
+      <c r="G144" s="97" t="n"/>
       <c r="H144" s="24" t="n"/>
-      <c r="I144" s="96" t="n"/>
+      <c r="I144" s="98" t="n"/>
       <c r="J144" s="26" t="n">
         <v>1</v>
       </c>
@@ -47855,9 +47893,9 @@
       <c r="D145" s="22" t="n"/>
       <c r="E145" s="22" t="n"/>
       <c r="F145" s="28" t="n"/>
-      <c r="G145" s="95" t="n"/>
+      <c r="G145" s="97" t="n"/>
       <c r="H145" s="24" t="n"/>
-      <c r="I145" s="96" t="n"/>
+      <c r="I145" s="98" t="n"/>
       <c r="J145" s="26" t="n">
         <v>1</v>
       </c>
@@ -47880,9 +47918,9 @@
       <c r="D146" s="22" t="n"/>
       <c r="E146" s="22" t="n"/>
       <c r="F146" s="28" t="n"/>
-      <c r="G146" s="95" t="n"/>
+      <c r="G146" s="97" t="n"/>
       <c r="H146" s="24" t="n"/>
-      <c r="I146" s="96" t="n"/>
+      <c r="I146" s="98" t="n"/>
       <c r="J146" s="26" t="n">
         <v>1</v>
       </c>
@@ -47905,9 +47943,9 @@
       <c r="D147" s="22" t="n"/>
       <c r="E147" s="22" t="n"/>
       <c r="F147" s="28" t="n"/>
-      <c r="G147" s="95" t="n"/>
+      <c r="G147" s="97" t="n"/>
       <c r="H147" s="24" t="n"/>
-      <c r="I147" s="96" t="n"/>
+      <c r="I147" s="98" t="n"/>
       <c r="J147" s="26" t="n">
         <v>1</v>
       </c>
@@ -47930,9 +47968,9 @@
       <c r="D148" s="22" t="n"/>
       <c r="E148" s="22" t="n"/>
       <c r="F148" s="28" t="n"/>
-      <c r="G148" s="95" t="n"/>
+      <c r="G148" s="97" t="n"/>
       <c r="H148" s="24" t="n"/>
-      <c r="I148" s="96" t="n"/>
+      <c r="I148" s="98" t="n"/>
       <c r="J148" s="26" t="n">
         <v>1</v>
       </c>
@@ -47955,9 +47993,9 @@
       <c r="D149" s="22" t="n"/>
       <c r="E149" s="22" t="n"/>
       <c r="F149" s="28" t="n"/>
-      <c r="G149" s="95" t="n"/>
+      <c r="G149" s="97" t="n"/>
       <c r="H149" s="24" t="n"/>
-      <c r="I149" s="96" t="n"/>
+      <c r="I149" s="98" t="n"/>
       <c r="J149" s="26" t="n">
         <v>1</v>
       </c>
@@ -47980,9 +48018,9 @@
       <c r="D150" s="22" t="n"/>
       <c r="E150" s="22" t="n"/>
       <c r="F150" s="28" t="n"/>
-      <c r="G150" s="95" t="n"/>
+      <c r="G150" s="97" t="n"/>
       <c r="H150" s="24" t="n"/>
-      <c r="I150" s="96" t="n"/>
+      <c r="I150" s="98" t="n"/>
       <c r="J150" s="26" t="n">
         <v>1</v>
       </c>
@@ -48005,9 +48043,9 @@
       <c r="D151" s="22" t="n"/>
       <c r="E151" s="22" t="n"/>
       <c r="F151" s="28" t="n"/>
-      <c r="G151" s="95" t="n"/>
+      <c r="G151" s="97" t="n"/>
       <c r="H151" s="24" t="n"/>
-      <c r="I151" s="96" t="n"/>
+      <c r="I151" s="98" t="n"/>
       <c r="J151" s="26" t="n">
         <v>1</v>
       </c>
@@ -48030,9 +48068,9 @@
       <c r="D152" s="22" t="n"/>
       <c r="E152" s="22" t="n"/>
       <c r="F152" s="28" t="n"/>
-      <c r="G152" s="95" t="n"/>
+      <c r="G152" s="97" t="n"/>
       <c r="H152" s="24" t="n"/>
-      <c r="I152" s="96" t="n"/>
+      <c r="I152" s="98" t="n"/>
       <c r="J152" s="26" t="n">
         <v>1</v>
       </c>
@@ -48055,9 +48093,9 @@
       <c r="D153" s="22" t="n"/>
       <c r="E153" s="22" t="n"/>
       <c r="F153" s="28" t="n"/>
-      <c r="G153" s="95" t="n"/>
+      <c r="G153" s="97" t="n"/>
       <c r="H153" s="24" t="n"/>
-      <c r="I153" s="96" t="n"/>
+      <c r="I153" s="98" t="n"/>
       <c r="J153" s="26" t="n">
         <v>1</v>
       </c>
@@ -48080,9 +48118,9 @@
       <c r="D154" s="22" t="n"/>
       <c r="E154" s="22" t="n"/>
       <c r="F154" s="28" t="n"/>
-      <c r="G154" s="95" t="n"/>
+      <c r="G154" s="97" t="n"/>
       <c r="H154" s="24" t="n"/>
-      <c r="I154" s="96" t="n"/>
+      <c r="I154" s="98" t="n"/>
       <c r="J154" s="26" t="n">
         <v>1</v>
       </c>
@@ -48105,9 +48143,9 @@
       <c r="D155" s="22" t="n"/>
       <c r="E155" s="22" t="n"/>
       <c r="F155" s="28" t="n"/>
-      <c r="G155" s="95" t="n"/>
+      <c r="G155" s="97" t="n"/>
       <c r="H155" s="24" t="n"/>
-      <c r="I155" s="96" t="n"/>
+      <c r="I155" s="98" t="n"/>
       <c r="J155" s="26" t="n">
         <v>1</v>
       </c>
@@ -48130,9 +48168,9 @@
       <c r="D156" s="59" t="n"/>
       <c r="E156" s="59" t="n"/>
       <c r="F156" s="71" t="n"/>
-      <c r="G156" s="95" t="n"/>
+      <c r="G156" s="97" t="n"/>
       <c r="H156" s="73" t="n"/>
-      <c r="I156" s="96" t="n"/>
+      <c r="I156" s="98" t="n"/>
       <c r="J156" s="26" t="n">
         <v>1</v>
       </c>

</xml_diff>